<commit_message>
update Kompetenzraster Python Teil
</commit_message>
<xml_diff>
--- a/files/MCQs.xlsx
+++ b/files/MCQs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39AB3D14-A4B6-DD47-9E7B-86BC68624636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A846D8C8-FC02-5840-A028-A4C25BAB7F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="3261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="3262">
   <si>
     <t>Approved</t>
   </si>
@@ -9827,6 +9827,9 @@
   </si>
   <si>
     <t>Python erlaubt keine Sonderzeichen wie '@' oder '%' innerhalb von Variablennamen. Diese sind in Variablennamen nicht zulässig.</t>
+  </si>
+  <si>
+    <t>Tupel</t>
   </si>
 </sst>
 </file>
@@ -27685,10 +27688,10 @@
         <v>39</v>
       </c>
       <c r="E178" t="s">
-        <v>2245</v>
+        <v>3261</v>
       </c>
       <c r="F178">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G178" t="s">
         <v>2285</v>
@@ -28472,7 +28475,7 @@
         <v>2391</v>
       </c>
       <c r="F186">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G186" t="s">
         <v>2392</v>
@@ -28570,7 +28573,7 @@
         <v>2391</v>
       </c>
       <c r="F187">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G187" t="s">
         <v>2401</v>

</xml_diff>

<commit_message>
do not run old seedMCQ
</commit_message>
<xml_diff>
--- a/files/MCQs.xlsx
+++ b/files/MCQs.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E5F065-4398-3145-9545-E58D7C7311D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9E2BC9-9509-3042-845B-9FD110941BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="30240" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evaluation" sheetId="1" r:id="rId1"/>
@@ -22868,7 +22868,7 @@
         <v>1153</v>
       </c>
       <c r="F155">
-        <v>206</v>
+        <v>85</v>
       </c>
       <c r="G155" t="s">
         <v>1523</v>
@@ -22967,7 +22967,7 @@
         <v>1153</v>
       </c>
       <c r="F156">
-        <v>206</v>
+        <v>85</v>
       </c>
       <c r="G156" t="s">
         <v>1531</v>
@@ -23065,7 +23065,7 @@
         <v>1153</v>
       </c>
       <c r="F157">
-        <v>206</v>
+        <v>85</v>
       </c>
       <c r="G157" t="s">
         <v>1544</v>

</xml_diff>